<commit_message>
결과 파일 업데이트 2026-08-11 09:03
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260811.xlsx
+++ b/results/andar_할인율모니터링_20260811.xlsx
@@ -733,12 +733,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2,173</t>
+          <t>2,174</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>4,758</t>
+          <t>4,759</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>67,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>54,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1825,12 +1825,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1867,22 +1867,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>33,000</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>200</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2035,12 +2035,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>64,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2203,12 +2203,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2371,12 +2371,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>63,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>240</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>44,000</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>191</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2707,12 +2707,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>4,758</t>
+          <t>4,759</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2791,12 +2791,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3001,12 +3001,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3421,12 +3421,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>1,054</t>
+          <t>1,055</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2,994</t>
+          <t>2,995</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2,994</t>
+          <t>2,995</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3757,12 +3757,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>93,000</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3841,12 +3841,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>63,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4177,12 +4177,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>67,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>532</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>532</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">

</xml_diff>